<commit_message>
gamma per arc by transport mode (node 44 included)
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/gamma_defined_per_arc_pipeline.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/gamma_defined_per_arc_pipeline.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR44"/>
+  <dimension ref="A1:AS45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,6 +561,9 @@
       <c r="AR1" s="1" t="n">
         <v>43</v>
       </c>
+      <c r="AS1" s="1" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -573,7 +576,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>11593775.784</v>
+        <v>20725826.022</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -693,6 +696,9 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -728,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>22587167.895</v>
+        <v>43057180.63</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -827,6 +833,9 @@
         <v>0</v>
       </c>
       <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -853,13 +862,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>10009170.249</v>
+        <v>11111337.052</v>
       </c>
       <c r="I4" t="n">
-        <v>8568719.527000001</v>
+        <v>9374947.4</v>
       </c>
       <c r="J4" t="n">
-        <v>9928247.164999999</v>
+        <v>11259128.566</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -961,6 +970,9 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -981,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>3482583.828</v>
+        <v>4801455.485</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -999,10 +1011,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>7677831.062</v>
+        <v>14472504.464</v>
       </c>
       <c r="M5" t="n">
-        <v>10416381.589</v>
+        <v>17632236.782</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -1095,6 +1107,9 @@
         <v>0</v>
       </c>
       <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1118,7 +1133,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>6448665.562</v>
+        <v>9529119.721000001</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1133,10 +1148,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>6930490.158</v>
+        <v>11642916.786</v>
       </c>
       <c r="M6" t="n">
-        <v>9152901.341</v>
+        <v>14447067.671</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1229,6 +1244,9 @@
         <v>0</v>
       </c>
       <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1255,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>3949812.122</v>
+        <v>4941762.442</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1270,10 +1288,10 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>6534473.007</v>
+        <v>11297084.464</v>
       </c>
       <c r="N7" t="n">
-        <v>4650726.623</v>
+        <v>6930708.091</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -1363,6 +1381,9 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1392,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>4206781.643</v>
+        <v>4848259.473</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -1407,16 +1428,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>5427848.161</v>
+        <v>7574350.7</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>8597549.301999999</v>
+        <v>11577246.415</v>
       </c>
       <c r="Q8" t="n">
-        <v>10822178.52</v>
+        <v>12252775.946</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1497,6 +1518,9 @@
         <v>0</v>
       </c>
       <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1529,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>5341911.006</v>
+        <v>5965737.115</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1541,16 +1565,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>7260974.12</v>
+        <v>8885480.777000001</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>8757520.844000001</v>
+        <v>10923692.194</v>
       </c>
       <c r="Q9" t="n">
-        <v>9637348.645</v>
+        <v>11287538.739</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1631,6 +1655,9 @@
         <v>0</v>
       </c>
       <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1666,7 +1693,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>11567162.042</v>
+        <v>19315754.459</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1681,10 +1708,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>9550851.914999999</v>
+        <v>11234613.437</v>
       </c>
       <c r="Q10" t="n">
-        <v>8257793.615</v>
+        <v>9284653.771</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1696,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>13371738.559</v>
+        <v>17246111.729</v>
       </c>
       <c r="V10" t="n">
-        <v>15902092.76</v>
+        <v>26220602.194</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -1765,6 +1792,9 @@
         <v>0</v>
       </c>
       <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1833,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>14122820.527</v>
+        <v>27046672.051</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -1899,6 +1929,9 @@
         <v>0</v>
       </c>
       <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1940,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>4569565.532</v>
+        <v>9775222.384</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1955,10 +1988,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>5413732.136</v>
+        <v>10472449.158</v>
       </c>
       <c r="S12" t="n">
-        <v>7216637.748</v>
+        <v>13960677.761</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -2033,6 +2066,9 @@
         <v>0</v>
       </c>
       <c r="AR12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2080,7 +2116,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>3015508.227</v>
+        <v>6484911.455</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -2092,7 +2128,7 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>5227002.481</v>
+        <v>11090227.769</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -2167,6 +2203,9 @@
         <v>0</v>
       </c>
       <c r="AR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2214,10 +2253,10 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>3771438.312</v>
+        <v>7790816.599</v>
       </c>
       <c r="P14" t="n">
-        <v>5033853.667</v>
+        <v>8975228.963</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -2301,6 +2340,9 @@
         <v>0</v>
       </c>
       <c r="AR14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2351,7 +2393,7 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>4347955.574</v>
+        <v>8894438.436000001</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -2363,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>7070702.592</v>
+        <v>13124905.624</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -2375,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>14535688.748</v>
+        <v>20982900.717</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -2435,6 +2477,9 @@
         <v>0</v>
       </c>
       <c r="AR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2488,7 +2533,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>5540879.744</v>
+        <v>6288574.633</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -2500,7 +2545,7 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>10451881.53</v>
+        <v>12344581.731</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
@@ -2509,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>14154436.886</v>
+        <v>18159647.818</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -2569,6 +2614,9 @@
         <v>0</v>
       </c>
       <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2634,7 +2682,7 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>7323094.295</v>
+        <v>8495935.429</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -2703,6 +2751,9 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2762,7 +2813,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>4477751.815</v>
+        <v>8801282.557</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -2837,6 +2888,9 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2884,7 +2938,7 @@
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>5534641.087</v>
+        <v>10913107.797</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -2899,7 +2953,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>3473528.167</v>
+        <v>6651378.626</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -2971,6 +3025,9 @@
         <v>0</v>
       </c>
       <c r="AR19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3036,16 +3093,16 @@
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>12544180.965</v>
+        <v>15571488.382</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>7974339.159</v>
+        <v>15310138.6</v>
       </c>
       <c r="X20" t="n">
-        <v>9897418.574999999</v>
+        <v>14588274.417</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -3105,6 +3162,9 @@
         <v>0</v>
       </c>
       <c r="AR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3179,16 +3239,16 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>12541828.081</v>
+        <v>14951711.211</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>10956484.755</v>
+        <v>12777354.246</v>
       </c>
       <c r="AA21" t="n">
-        <v>21371149.789</v>
+        <v>25659160.493</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>
@@ -3197,7 +3257,7 @@
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>27603974</v>
+        <v>0</v>
       </c>
       <c r="AE21" t="n">
         <v>0</v>
@@ -3206,7 +3266,7 @@
         <v>0</v>
       </c>
       <c r="AG21" t="n">
-        <v>29188170.814</v>
+        <v>0</v>
       </c>
       <c r="AH21" t="n">
         <v>0</v>
@@ -3240,6 +3300,9 @@
       </c>
       <c r="AR21" t="n">
         <v>0</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>16606349.112</v>
       </c>
     </row>
     <row r="22">
@@ -3304,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>5039819.163</v>
+        <v>7530702.863</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -3319,7 +3382,7 @@
         <v>0</v>
       </c>
       <c r="Z22" t="n">
-        <v>9241520.153000001</v>
+        <v>14500828.738</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
@@ -3373,6 +3436,9 @@
         <v>0</v>
       </c>
       <c r="AR22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3438,7 +3504,7 @@
         <v>7974339.159</v>
       </c>
       <c r="U23" t="n">
-        <v>15466715.625</v>
+        <v>19747328.541</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -3447,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>6097886.112</v>
+        <v>10922632.506</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -3507,6 +3573,9 @@
         <v>0</v>
       </c>
       <c r="AR23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3584,7 +3653,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>3019274.436</v>
+        <v>5346379.34</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
@@ -3641,6 +3710,9 @@
         <v>0</v>
       </c>
       <c r="AR24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3721,13 +3793,13 @@
         <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>14419978.42</v>
+        <v>17371958.526</v>
       </c>
       <c r="AA25" t="n">
-        <v>11304021.22</v>
+        <v>16862932.58</v>
       </c>
       <c r="AB25" t="n">
-        <v>20209492.332</v>
+        <v>0</v>
       </c>
       <c r="AC25" t="n">
         <v>0</v>
@@ -3776,6 +3848,9 @@
       </c>
       <c r="AR25" t="n">
         <v>0</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>17010654.819</v>
       </c>
     </row>
     <row r="26">
@@ -3858,16 +3933,16 @@
         <v>0</v>
       </c>
       <c r="AA26" t="n">
-        <v>16151380.769</v>
+        <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>10253712.677</v>
+        <v>11887336.562</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>18158286.849</v>
+        <v>20135237.566</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -3876,7 +3951,7 @@
         <v>0</v>
       </c>
       <c r="AG26" t="n">
-        <v>20757607.265</v>
+        <v>0</v>
       </c>
       <c r="AH26" t="n">
         <v>0</v>
@@ -3910,6 +3985,9 @@
       </c>
       <c r="AR26" t="n">
         <v>0</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>6286914.042</v>
       </c>
     </row>
     <row r="27">
@@ -3995,28 +4073,28 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>15922645.239</v>
+        <v>18226518.646</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>13911725.292</v>
+        <v>16195261.047</v>
       </c>
       <c r="AE27" t="n">
-        <v>19407946.639</v>
+        <v>23013899.923</v>
       </c>
       <c r="AF27" t="n">
-        <v>11528325.606</v>
+        <v>14736605.761</v>
       </c>
       <c r="AG27" t="n">
-        <v>12704555.447</v>
+        <v>14468978.655</v>
       </c>
       <c r="AH27" t="n">
         <v>0</v>
       </c>
       <c r="AI27" t="n">
-        <v>13320592.542</v>
+        <v>17571312.2</v>
       </c>
       <c r="AJ27" t="n">
         <v>0</v>
@@ -4044,6 +4122,9 @@
       </c>
       <c r="AR27" t="n">
         <v>0</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>13900223.769</v>
       </c>
     </row>
     <row r="28">
@@ -4135,10 +4216,10 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>10706103.428</v>
+        <v>11723950.81</v>
       </c>
       <c r="AE28" t="n">
-        <v>9190862.503</v>
+        <v>12095805.123</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
@@ -4177,6 +4258,9 @@
         <v>0</v>
       </c>
       <c r="AR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4260,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>22938271.785</v>
+        <v>42863877.014</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -4281,10 +4365,10 @@
         <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>16268576.558</v>
+        <v>30631832.97</v>
       </c>
       <c r="AI29" t="n">
-        <v>24024112.173</v>
+        <v>41321354.793</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -4311,6 +4395,9 @@
         <v>0</v>
       </c>
       <c r="AR29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4406,13 +4493,13 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>8414252.550000001</v>
+        <v>9645032.526000001</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
       </c>
       <c r="AG30" t="n">
-        <v>5218473.715</v>
+        <v>5653504.381</v>
       </c>
       <c r="AH30" t="n">
         <v>0</v>
@@ -4421,13 +4508,13 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>16138216.371</v>
+        <v>17656215.019</v>
       </c>
       <c r="AK30" t="n">
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>14025835.936</v>
+        <v>15413974.664</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
@@ -4445,6 +4532,9 @@
         <v>0</v>
       </c>
       <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4555,13 +4645,13 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>12386749.84</v>
+        <v>15002116.384</v>
       </c>
       <c r="AK31" t="n">
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>12169450.76</v>
+        <v>13850255.241</v>
       </c>
       <c r="AM31" t="n">
         <v>0</v>
@@ -4579,6 +4669,9 @@
         <v>0</v>
       </c>
       <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4680,13 +4773,13 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
-        <v>5223805.445</v>
+        <v>6035405.064</v>
       </c>
       <c r="AH32" t="n">
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>5364717.35</v>
+        <v>7815207.91</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -4695,7 +4788,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>19110831.517</v>
+        <v>21383688.006</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -4713,6 +4806,9 @@
         <v>0</v>
       </c>
       <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4829,7 +4925,7 @@
         <v>0</v>
       </c>
       <c r="AL33" t="n">
-        <v>15933925.509</v>
+        <v>17221705.652</v>
       </c>
       <c r="AM33" t="n">
         <v>0</v>
@@ -4847,6 +4943,9 @@
         <v>0</v>
       </c>
       <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4954,19 +5053,19 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
-        <v>10702994.644</v>
+        <v>14840099.291</v>
       </c>
       <c r="AJ34" t="n">
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>6209624.441</v>
+        <v>9077992.708000001</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
       </c>
       <c r="AM34" t="n">
-        <v>11355430.375</v>
+        <v>16428666.588</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -4981,6 +5080,9 @@
         <v>0</v>
       </c>
       <c r="AR34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5100,7 +5202,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="n">
-        <v>6597327.838</v>
+        <v>10265354.688</v>
       </c>
       <c r="AN35" t="n">
         <v>0</v>
@@ -5115,6 +5217,9 @@
         <v>0</v>
       </c>
       <c r="AR35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5231,7 +5336,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>5053987.316</v>
+        <v>5628128.291</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -5240,7 +5345,7 @@
         <v>0</v>
       </c>
       <c r="AO36" t="n">
-        <v>10445117.557</v>
+        <v>16696109.511</v>
       </c>
       <c r="AP36" t="n">
         <v>0</v>
@@ -5249,6 +5354,9 @@
         <v>0</v>
       </c>
       <c r="AR36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5356,7 +5464,7 @@
         <v>6209624.441</v>
       </c>
       <c r="AI37" t="n">
-        <v>10718382.193</v>
+        <v>13689891.675</v>
       </c>
       <c r="AJ37" t="n">
         <v>0</v>
@@ -5368,7 +5476,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="n">
-        <v>8761740.629000001</v>
+        <v>12719385.223</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -5383,6 +5491,9 @@
         <v>0</v>
       </c>
       <c r="AR37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5514,9 +5625,12 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
-        <v>4449736.075</v>
+        <v>5186532.415</v>
       </c>
       <c r="AR38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5653,6 +5767,9 @@
       <c r="AR39" t="n">
         <v>0</v>
       </c>
+      <c r="AS39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -5764,13 +5881,13 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
-        <v>10772694.722</v>
+        <v>17544317.781</v>
       </c>
       <c r="AL40" t="n">
         <v>0</v>
       </c>
       <c r="AM40" t="n">
-        <v>17147347.112</v>
+        <v>21273343.257</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -5785,6 +5902,9 @@
         <v>0</v>
       </c>
       <c r="AR40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5901,7 +6021,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>11571041.404</v>
+        <v>15185780.988</v>
       </c>
       <c r="AM41" t="n">
         <v>0</v>
@@ -5919,6 +6039,9 @@
         <v>0</v>
       </c>
       <c r="AR41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6032,13 +6155,13 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
-        <v>22957541.853</v>
+        <v>26070312.183</v>
       </c>
       <c r="AL42" t="n">
         <v>0</v>
       </c>
       <c r="AM42" t="n">
-        <v>22490477.157</v>
+        <v>23700399.371</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
@@ -6053,6 +6176,9 @@
         <v>0</v>
       </c>
       <c r="AR42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6187,7 +6313,10 @@
         <v>0</v>
       </c>
       <c r="AR43" t="n">
-        <v>2953413.162</v>
+        <v>3042015.556</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -6321,6 +6450,146 @@
         <v>0</v>
       </c>
       <c r="AR44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>5441450.231</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>9687115.025</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>15950315.116</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6335,7 +6604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR44"/>
+  <dimension ref="A1:AS45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6468,6 +6737,9 @@
       <c r="AR1" s="1" t="n">
         <v>43</v>
       </c>
+      <c r="AS1" s="1" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -6480,7 +6752,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>238849.751</v>
+        <v>396836.255</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -6600,6 +6872,9 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6635,7 +6910,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>386729.821</v>
+        <v>676760.808</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -6734,6 +7009,9 @@
         <v>0</v>
       </c>
       <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6760,13 +7038,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>203858.358</v>
+        <v>223685.926</v>
       </c>
       <c r="I4" t="n">
-        <v>184401.515</v>
+        <v>200033.479</v>
       </c>
       <c r="J4" t="n">
-        <v>216480.259</v>
+        <v>242224.784</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -6868,6 +7146,9 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6888,7 +7169,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>133149.791</v>
+        <v>176842.288</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -6906,10 +7187,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>173983.765</v>
+        <v>304159.013</v>
       </c>
       <c r="M5" t="n">
-        <v>216008.198</v>
+        <v>341784.483</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -7002,6 +7283,9 @@
         <v>0</v>
       </c>
       <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7025,7 +7309,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>152806.266</v>
+        <v>215126.677</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -7040,10 +7324,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>159438.167</v>
+        <v>251775.852</v>
       </c>
       <c r="M6" t="n">
-        <v>190922.245</v>
+        <v>284064.136</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -7136,6 +7420,9 @@
         <v>0</v>
       </c>
       <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7162,7 +7449,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>139835.638</v>
+        <v>170867.185</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -7177,10 +7464,10 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>154168.234</v>
+        <v>249986.237</v>
       </c>
       <c r="N7" t="n">
-        <v>162709.634</v>
+        <v>231461.651</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -7270,6 +7557,9 @@
         <v>0</v>
       </c>
       <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7299,7 +7589,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>153257.355</v>
+        <v>174787.935</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -7314,16 +7604,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>161661.065</v>
+        <v>217472.309</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>184660.078</v>
+        <v>239420.551</v>
       </c>
       <c r="Q8" t="n">
-        <v>228959.434</v>
+        <v>256304.465</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -7404,6 +7694,9 @@
         <v>0</v>
       </c>
       <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7436,7 +7729,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>151975.818</v>
+        <v>167892.99</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -7448,16 +7741,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>171056.695</v>
+        <v>205091.481</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>186745.15</v>
+        <v>227076.685</v>
       </c>
       <c r="Q9" t="n">
-        <v>202491.376</v>
+        <v>232682.486</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -7538,6 +7831,9 @@
         <v>0</v>
       </c>
       <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7573,7 +7869,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>242960.938</v>
+        <v>379760.435</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -7588,10 +7884,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>201185.096</v>
+        <v>233404.831</v>
       </c>
       <c r="Q10" t="n">
-        <v>190883.397</v>
+        <v>212235.556</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -7603,10 +7899,10 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>256335.138</v>
+        <v>319952.724</v>
       </c>
       <c r="V10" t="n">
-        <v>288264.261</v>
+        <v>444151.591</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -7672,6 +7968,9 @@
         <v>0</v>
       </c>
       <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7740,7 +8039,7 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>282166.137</v>
+        <v>497371.661</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -7806,6 +8105,9 @@
         <v>0</v>
       </c>
       <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7847,7 +8149,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>168488.747</v>
+        <v>332512.107</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -7862,10 +8164,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>160286.536</v>
+        <v>288184.843</v>
       </c>
       <c r="S12" t="n">
-        <v>170767.418</v>
+        <v>305926.415</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -7940,6 +8242,9 @@
         <v>0</v>
       </c>
       <c r="AR12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7987,7 +8292,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>133778.092</v>
+        <v>266135.957</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -7999,7 +8304,7 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>163654.392</v>
+        <v>319638.71</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -8074,6 +8379,9 @@
         <v>0</v>
       </c>
       <c r="AR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8121,10 +8429,10 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>141530.392</v>
+        <v>270786.575</v>
       </c>
       <c r="P14" t="n">
-        <v>152309.793</v>
+        <v>254905.38</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -8208,6 +8516,9 @@
         <v>0</v>
       </c>
       <c r="AR14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8258,7 +8569,7 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>146995.013</v>
+        <v>278679.533</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -8270,7 +8581,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>159526.24</v>
+        <v>275039.345</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -8282,7 +8593,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>276458.878</v>
+        <v>381365.795</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -8342,6 +8653,9 @@
         <v>0</v>
       </c>
       <c r="AR15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8395,7 +8709,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>166455.535</v>
+        <v>186910.71</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -8407,7 +8721,7 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>216403.495</v>
+        <v>251513.631</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
@@ -8416,7 +8730,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>282691.703</v>
+        <v>351062.91</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -8476,6 +8790,9 @@
         <v>0</v>
       </c>
       <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8541,7 +8858,7 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>158599.463</v>
+        <v>181067.282</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -8610,6 +8927,9 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8669,7 +8989,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>156723.072</v>
+        <v>286108.794</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -8744,6 +9064,9 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8791,7 +9114,7 @@
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>160510.736</v>
+        <v>294160.571</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -8806,7 +9129,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>132736.25</v>
+        <v>236369.709</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -8878,6 +9201,9 @@
         <v>0</v>
       </c>
       <c r="AR19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8943,16 +9269,16 @@
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>265902.931</v>
+        <v>323337.953</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>168587.082</v>
+        <v>299034.074</v>
       </c>
       <c r="X20" t="n">
-        <v>215998.484</v>
+        <v>302925.872</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -9012,6 +9338,9 @@
         <v>0</v>
       </c>
       <c r="AR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9086,16 +9415,16 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>256733.485</v>
+        <v>300346.43</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>240120.499</v>
+        <v>275595.844</v>
       </c>
       <c r="AA21" t="n">
-        <v>369480.611</v>
+        <v>435008.9</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>
@@ -9104,7 +9433,7 @@
         <v>0</v>
       </c>
       <c r="AD21" t="n">
-        <v>448543.355</v>
+        <v>0</v>
       </c>
       <c r="AE21" t="n">
         <v>0</v>
@@ -9113,7 +9442,7 @@
         <v>0</v>
       </c>
       <c r="AG21" t="n">
-        <v>471921.04</v>
+        <v>0</v>
       </c>
       <c r="AH21" t="n">
         <v>0</v>
@@ -9147,6 +9476,9 @@
       </c>
       <c r="AR21" t="n">
         <v>0</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>310322.394</v>
       </c>
     </row>
     <row r="22">
@@ -9211,7 +9543,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>174224.308</v>
+        <v>248070.676</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -9226,7 +9558,7 @@
         <v>0</v>
       </c>
       <c r="Z22" t="n">
-        <v>184520.172</v>
+        <v>273099.537</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
@@ -9280,6 +9612,9 @@
         <v>0</v>
       </c>
       <c r="AR22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9345,7 +9680,7 @@
         <v>168587.082</v>
       </c>
       <c r="U23" t="n">
-        <v>279941.512</v>
+        <v>347201.175</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -9354,7 +9689,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>159563.609</v>
+        <v>266646.859</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -9414,6 +9749,9 @@
         <v>0</v>
       </c>
       <c r="AR23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9491,7 +9829,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>135586.899</v>
+        <v>225775.014</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
@@ -9548,6 +9886,9 @@
         <v>0</v>
       </c>
       <c r="AR24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9628,13 +9969,13 @@
         <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>275936.202</v>
+        <v>324566.089</v>
       </c>
       <c r="AA25" t="n">
-        <v>241384.095</v>
+        <v>342708.225</v>
       </c>
       <c r="AB25" t="n">
-        <v>354132.529</v>
+        <v>0</v>
       </c>
       <c r="AC25" t="n">
         <v>0</v>
@@ -9683,6 +10024,9 @@
       </c>
       <c r="AR25" t="n">
         <v>0</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>315423.399</v>
       </c>
     </row>
     <row r="26">
@@ -9765,16 +10109,16 @@
         <v>0</v>
       </c>
       <c r="AA26" t="n">
-        <v>284902.939</v>
+        <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>217690.091</v>
+        <v>248859.702</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>331992.35</v>
+        <v>364919.482</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -9783,7 +10127,7 @@
         <v>0</v>
       </c>
       <c r="AG26" t="n">
-        <v>361678.367</v>
+        <v>0</v>
       </c>
       <c r="AH26" t="n">
         <v>0</v>
@@ -9817,6 +10161,9 @@
       </c>
       <c r="AR26" t="n">
         <v>0</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>193229.253</v>
       </c>
     </row>
     <row r="27">
@@ -9902,28 +10249,28 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>288320.936</v>
+        <v>325434.931</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>277638.469</v>
+        <v>318693.35</v>
       </c>
       <c r="AE27" t="n">
-        <v>353702.197</v>
+        <v>411300.821</v>
       </c>
       <c r="AF27" t="n">
-        <v>242664.932</v>
+        <v>300326.36</v>
       </c>
       <c r="AG27" t="n">
-        <v>253576.153</v>
+        <v>284856.764</v>
       </c>
       <c r="AH27" t="n">
         <v>0</v>
       </c>
       <c r="AI27" t="n">
-        <v>268357.874</v>
+        <v>342066.528</v>
       </c>
       <c r="AJ27" t="n">
         <v>0</v>
@@ -9951,6 +10298,9 @@
       </c>
       <c r="AR27" t="n">
         <v>0</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>291864.947</v>
       </c>
     </row>
     <row r="28">
@@ -10042,10 +10392,10 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>226882.206</v>
+        <v>246328.323</v>
       </c>
       <c r="AE28" t="n">
-        <v>184035.706</v>
+        <v>234014.031</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
@@ -10084,6 +10434,9 @@
         <v>0</v>
       </c>
       <c r="AR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10167,7 +10520,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>401650.314</v>
+        <v>691020.8100000001</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -10188,10 +10541,10 @@
         <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>285665.201</v>
+        <v>494395.23</v>
       </c>
       <c r="AI29" t="n">
-        <v>414195.008</v>
+        <v>664412.25</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -10218,6 +10571,9 @@
         <v>0</v>
       </c>
       <c r="AR29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10313,13 +10669,13 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>186278.964</v>
+        <v>211175.566</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
       </c>
       <c r="AG30" t="n">
-        <v>161153.811</v>
+        <v>174063.459</v>
       </c>
       <c r="AH30" t="n">
         <v>0</v>
@@ -10328,13 +10684,13 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>302752.959</v>
+        <v>330174.219</v>
       </c>
       <c r="AK30" t="n">
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>280195.435</v>
+        <v>305286.359</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
@@ -10352,6 +10708,9 @@
         <v>0</v>
       </c>
       <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10462,13 +10821,13 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>247357.413</v>
+        <v>293208.677</v>
       </c>
       <c r="AK31" t="n">
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>249679.454</v>
+        <v>280969.489</v>
       </c>
       <c r="AM31" t="n">
         <v>0</v>
@@ -10486,6 +10845,9 @@
         <v>0</v>
       </c>
       <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10587,13 +10949,13 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
-        <v>163611.695</v>
+        <v>186156.717</v>
       </c>
       <c r="AH32" t="n">
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>152231.264</v>
+        <v>212238.573</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -10602,7 +10964,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>349574.709</v>
+        <v>386527.229</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -10620,6 +10982,9 @@
         <v>0</v>
       </c>
       <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10736,7 +11101,7 @@
         <v>0</v>
       </c>
       <c r="AL33" t="n">
-        <v>288356.891</v>
+        <v>309869.527</v>
       </c>
       <c r="AM33" t="n">
         <v>0</v>
@@ -10754,6 +11119,9 @@
         <v>0</v>
       </c>
       <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10861,19 +11229,19 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
-        <v>224945.228</v>
+        <v>299817.779</v>
       </c>
       <c r="AJ34" t="n">
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>147428.998</v>
+        <v>205147.596</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
       </c>
       <c r="AM34" t="n">
-        <v>241129.43</v>
+        <v>332903.751</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -10888,6 +11256,9 @@
         <v>0</v>
       </c>
       <c r="AR34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11007,7 +11378,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="n">
-        <v>162309.229</v>
+        <v>240014.866</v>
       </c>
       <c r="AN35" t="n">
         <v>0</v>
@@ -11022,6 +11393,9 @@
         <v>0</v>
       </c>
       <c r="AR35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11138,7 +11512,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>152518.353</v>
+        <v>168505.557</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -11147,7 +11521,7 @@
         <v>0</v>
       </c>
       <c r="AO36" t="n">
-        <v>228094.92</v>
+        <v>343878.465</v>
       </c>
       <c r="AP36" t="n">
         <v>0</v>
@@ -11156,6 +11530,9 @@
         <v>0</v>
       </c>
       <c r="AR36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11263,7 +11640,7 @@
         <v>147428.998</v>
       </c>
       <c r="AI37" t="n">
-        <v>225324.218</v>
+        <v>279344.437</v>
       </c>
       <c r="AJ37" t="n">
         <v>0</v>
@@ -11275,7 +11652,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="n">
-        <v>186774.623</v>
+        <v>259417.902</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -11290,6 +11667,9 @@
         <v>0</v>
       </c>
       <c r="AR37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11421,9 +11801,12 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
-        <v>148406.882</v>
+        <v>170390.846</v>
       </c>
       <c r="AR38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11560,6 +11943,9 @@
       <c r="AR39" t="n">
         <v>0</v>
       </c>
+      <c r="AS39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -11671,13 +12057,13 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
-        <v>234785.519</v>
+        <v>359509.47</v>
       </c>
       <c r="AL40" t="n">
         <v>0</v>
       </c>
       <c r="AM40" t="n">
-        <v>306766.303</v>
+        <v>370480.205</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -11692,6 +12078,9 @@
         <v>0</v>
       </c>
       <c r="AR40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11808,7 +12197,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>242990.67</v>
+        <v>308187.102</v>
       </c>
       <c r="AM41" t="n">
         <v>0</v>
@@ -11826,6 +12215,9 @@
         <v>0</v>
       </c>
       <c r="AR41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11939,13 +12331,13 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
-        <v>392650.033</v>
+        <v>438126.995</v>
       </c>
       <c r="AL42" t="n">
         <v>0</v>
       </c>
       <c r="AM42" t="n">
-        <v>385117.054</v>
+        <v>402027.944</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
@@ -11960,6 +12352,9 @@
         <v>0</v>
       </c>
       <c r="AR42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12094,7 +12489,10 @@
         <v>0</v>
       </c>
       <c r="AR43" t="n">
-        <v>206868.548</v>
+        <v>213074.604</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -12228,6 +12626,146 @@
         <v>0</v>
       </c>
       <c r="AR44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>169474.854</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>211820.732</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>300453.543</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12242,7 +12780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR44"/>
+  <dimension ref="A1:AS45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12375,6 +12913,9 @@
       <c r="AR1" s="1" t="n">
         <v>43</v>
       </c>
+      <c r="AS1" s="1" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -12509,6 +13050,9 @@
       <c r="AR2" t="n">
         <v>0</v>
       </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -12643,6 +13187,9 @@
       <c r="AR3" t="n">
         <v>0</v>
       </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -12777,6 +13324,9 @@
       <c r="AR4" t="n">
         <v>0</v>
       </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -12911,6 +13461,9 @@
       <c r="AR5" t="n">
         <v>0</v>
       </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -13045,6 +13598,9 @@
       <c r="AR6" t="n">
         <v>0</v>
       </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -13179,6 +13735,9 @@
       <c r="AR7" t="n">
         <v>0</v>
       </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -13313,6 +13872,9 @@
       <c r="AR8" t="n">
         <v>0</v>
       </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -13447,6 +14009,9 @@
       <c r="AR9" t="n">
         <v>0</v>
       </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -13581,6 +14146,9 @@
       <c r="AR10" t="n">
         <v>0</v>
       </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -13715,6 +14283,9 @@
       <c r="AR11" t="n">
         <v>0</v>
       </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -13849,6 +14420,9 @@
       <c r="AR12" t="n">
         <v>0</v>
       </c>
+      <c r="AS12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -13983,6 +14557,9 @@
       <c r="AR13" t="n">
         <v>0</v>
       </c>
+      <c r="AS13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -14117,6 +14694,9 @@
       <c r="AR14" t="n">
         <v>0</v>
       </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -14251,6 +14831,9 @@
       <c r="AR15" t="n">
         <v>0</v>
       </c>
+      <c r="AS15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -14385,6 +14968,9 @@
       <c r="AR16" t="n">
         <v>0</v>
       </c>
+      <c r="AS16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -14519,6 +15105,9 @@
       <c r="AR17" t="n">
         <v>0</v>
       </c>
+      <c r="AS17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -14653,6 +15242,9 @@
       <c r="AR18" t="n">
         <v>0</v>
       </c>
+      <c r="AS18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -14787,6 +15379,9 @@
       <c r="AR19" t="n">
         <v>0</v>
       </c>
+      <c r="AS19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -14921,6 +15516,9 @@
       <c r="AR20" t="n">
         <v>0</v>
       </c>
+      <c r="AS20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -15055,6 +15653,9 @@
       <c r="AR21" t="n">
         <v>0</v>
       </c>
+      <c r="AS21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -15189,6 +15790,9 @@
       <c r="AR22" t="n">
         <v>0</v>
       </c>
+      <c r="AS22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -15323,6 +15927,9 @@
       <c r="AR23" t="n">
         <v>0</v>
       </c>
+      <c r="AS23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -15457,6 +16064,9 @@
       <c r="AR24" t="n">
         <v>0</v>
       </c>
+      <c r="AS24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -15591,6 +16201,9 @@
       <c r="AR25" t="n">
         <v>0</v>
       </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -15725,6 +16338,9 @@
       <c r="AR26" t="n">
         <v>0</v>
       </c>
+      <c r="AS26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -15859,6 +16475,9 @@
       <c r="AR27" t="n">
         <v>0</v>
       </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -15993,6 +16612,9 @@
       <c r="AR28" t="n">
         <v>0</v>
       </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -16127,6 +16749,9 @@
       <c r="AR29" t="n">
         <v>0</v>
       </c>
+      <c r="AS29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -16261,6 +16886,9 @@
       <c r="AR30" t="n">
         <v>0</v>
       </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -16395,6 +17023,9 @@
       <c r="AR31" t="n">
         <v>0</v>
       </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -16529,6 +17160,9 @@
       <c r="AR32" t="n">
         <v>0</v>
       </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -16663,6 +17297,9 @@
       <c r="AR33" t="n">
         <v>0</v>
       </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -16797,6 +17434,9 @@
       <c r="AR34" t="n">
         <v>0</v>
       </c>
+      <c r="AS34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -16931,6 +17571,9 @@
       <c r="AR35" t="n">
         <v>0</v>
       </c>
+      <c r="AS35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -17065,6 +17708,9 @@
       <c r="AR36" t="n">
         <v>0</v>
       </c>
+      <c r="AS36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -17199,6 +17845,9 @@
       <c r="AR37" t="n">
         <v>0</v>
       </c>
+      <c r="AS37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -17333,6 +17982,9 @@
       <c r="AR38" t="n">
         <v>0</v>
       </c>
+      <c r="AS38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -17467,6 +18119,9 @@
       <c r="AR39" t="n">
         <v>0</v>
       </c>
+      <c r="AS39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -17601,6 +18256,9 @@
       <c r="AR40" t="n">
         <v>0</v>
       </c>
+      <c r="AS40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -17735,6 +18393,9 @@
       <c r="AR41" t="n">
         <v>0</v>
       </c>
+      <c r="AS41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -17869,6 +18530,9 @@
       <c r="AR42" t="n">
         <v>0</v>
       </c>
+      <c r="AS42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -18003,6 +18667,9 @@
       <c r="AR43" t="n">
         <v>0</v>
       </c>
+      <c r="AS43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -18135,6 +18802,146 @@
         <v>0</v>
       </c>
       <c r="AR44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -18149,7 +18956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR44"/>
+  <dimension ref="A1:AS45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18282,6 +19089,9 @@
       <c r="AR1" s="1" t="n">
         <v>43</v>
       </c>
+      <c r="AS1" s="1" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -18416,6 +19226,9 @@
       <c r="AR2" t="n">
         <v>0</v>
       </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -18550,6 +19363,9 @@
       <c r="AR3" t="n">
         <v>0</v>
       </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -18684,6 +19500,9 @@
       <c r="AR4" t="n">
         <v>0</v>
       </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -18818,6 +19637,9 @@
       <c r="AR5" t="n">
         <v>0</v>
       </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -18952,6 +19774,9 @@
       <c r="AR6" t="n">
         <v>0</v>
       </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -19086,6 +19911,9 @@
       <c r="AR7" t="n">
         <v>0</v>
       </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -19220,6 +20048,9 @@
       <c r="AR8" t="n">
         <v>0</v>
       </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -19354,6 +20185,9 @@
       <c r="AR9" t="n">
         <v>0</v>
       </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -19488,6 +20322,9 @@
       <c r="AR10" t="n">
         <v>0</v>
       </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -19622,6 +20459,9 @@
       <c r="AR11" t="n">
         <v>0</v>
       </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -19756,6 +20596,9 @@
       <c r="AR12" t="n">
         <v>0</v>
       </c>
+      <c r="AS12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -19890,6 +20733,9 @@
       <c r="AR13" t="n">
         <v>0</v>
       </c>
+      <c r="AS13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -20024,6 +20870,9 @@
       <c r="AR14" t="n">
         <v>0</v>
       </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -20158,6 +21007,9 @@
       <c r="AR15" t="n">
         <v>0</v>
       </c>
+      <c r="AS15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -20292,6 +21144,9 @@
       <c r="AR16" t="n">
         <v>0</v>
       </c>
+      <c r="AS16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -20426,6 +21281,9 @@
       <c r="AR17" t="n">
         <v>0</v>
       </c>
+      <c r="AS17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -20560,6 +21418,9 @@
       <c r="AR18" t="n">
         <v>0</v>
       </c>
+      <c r="AS18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -20694,6 +21555,9 @@
       <c r="AR19" t="n">
         <v>0</v>
       </c>
+      <c r="AS19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -20828,6 +21692,9 @@
       <c r="AR20" t="n">
         <v>0</v>
       </c>
+      <c r="AS20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -20962,6 +21829,9 @@
       <c r="AR21" t="n">
         <v>0</v>
       </c>
+      <c r="AS21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -21096,6 +21966,9 @@
       <c r="AR22" t="n">
         <v>0</v>
       </c>
+      <c r="AS22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -21230,6 +22103,9 @@
       <c r="AR23" t="n">
         <v>0</v>
       </c>
+      <c r="AS23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -21364,6 +22240,9 @@
       <c r="AR24" t="n">
         <v>0</v>
       </c>
+      <c r="AS24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -21498,6 +22377,9 @@
       <c r="AR25" t="n">
         <v>0</v>
       </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -21632,6 +22514,9 @@
       <c r="AR26" t="n">
         <v>0</v>
       </c>
+      <c r="AS26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -21766,6 +22651,9 @@
       <c r="AR27" t="n">
         <v>0</v>
       </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -21900,6 +22788,9 @@
       <c r="AR28" t="n">
         <v>0</v>
       </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -22034,6 +22925,9 @@
       <c r="AR29" t="n">
         <v>0</v>
       </c>
+      <c r="AS29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -22168,6 +23062,9 @@
       <c r="AR30" t="n">
         <v>0</v>
       </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -22302,6 +23199,9 @@
       <c r="AR31" t="n">
         <v>0</v>
       </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -22436,6 +23336,9 @@
       <c r="AR32" t="n">
         <v>0</v>
       </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -22570,6 +23473,9 @@
       <c r="AR33" t="n">
         <v>0</v>
       </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -22704,6 +23610,9 @@
       <c r="AR34" t="n">
         <v>0</v>
       </c>
+      <c r="AS34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -22838,6 +23747,9 @@
       <c r="AR35" t="n">
         <v>0</v>
       </c>
+      <c r="AS35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -22972,6 +23884,9 @@
       <c r="AR36" t="n">
         <v>0</v>
       </c>
+      <c r="AS36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -23106,6 +24021,9 @@
       <c r="AR37" t="n">
         <v>0</v>
       </c>
+      <c r="AS37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -23240,6 +24158,9 @@
       <c r="AR38" t="n">
         <v>0</v>
       </c>
+      <c r="AS38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -23374,6 +24295,9 @@
       <c r="AR39" t="n">
         <v>0</v>
       </c>
+      <c r="AS39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -23508,6 +24432,9 @@
       <c r="AR40" t="n">
         <v>0</v>
       </c>
+      <c r="AS40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -23642,6 +24569,9 @@
       <c r="AR41" t="n">
         <v>0</v>
       </c>
+      <c r="AS41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -23776,6 +24706,9 @@
       <c r="AR42" t="n">
         <v>0</v>
       </c>
+      <c r="AS42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -23910,6 +24843,9 @@
       <c r="AR43" t="n">
         <v>0</v>
       </c>
+      <c r="AS43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -24042,6 +24978,146 @@
         <v>0</v>
       </c>
       <c r="AR44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS45" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added three classes of pipeline (small, medium, large) together with the analysis of the appropriate ranges
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/gamma_defined_per_arc_pipeline.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/gamma_defined_per_arc_pipeline.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="gamma1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="gamma2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="gamma3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="gamma4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,7 +576,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>20725826.022</v>
+        <v>42415003.756</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -734,7 +734,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>43057180.63</v>
+        <v>81276152.46799999</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -862,13 +862,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>11111337.052</v>
+        <v>23857676.3</v>
       </c>
       <c r="I4" t="n">
-        <v>9374947.4</v>
+        <v>20230040.131</v>
       </c>
       <c r="J4" t="n">
-        <v>11259128.566</v>
+        <v>24566107.257</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -993,7 +993,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>4801455.485</v>
+        <v>14218044.938</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1011,10 +1011,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>14472504.464</v>
+        <v>31333602.205</v>
       </c>
       <c r="M5" t="n">
-        <v>17632236.782</v>
+        <v>37172018.482</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -1133,7 +1133,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>9529119.721000001</v>
+        <v>21740369.21</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1148,10 +1148,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>11642916.786</v>
+        <v>27189578.781</v>
       </c>
       <c r="M6" t="n">
-        <v>14447067.671</v>
+        <v>31701988.748</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1273,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>4941762.442</v>
+        <v>12974409.435</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1288,10 +1288,10 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>11297084.464</v>
+        <v>23869017.067</v>
       </c>
       <c r="N7" t="n">
-        <v>6930708.091</v>
+        <v>17793207.158</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -1407,13 +1407,13 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>3949812.122</v>
+        <v>11730239.758</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>4848259.473</v>
+        <v>14628727.677</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -1428,16 +1428,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>7574350.7</v>
+        <v>20782775.394</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>11577246.415</v>
+        <v>26222534.69</v>
       </c>
       <c r="Q8" t="n">
-        <v>12252775.946</v>
+        <v>29830070.365</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1547,13 +1547,13 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>4206781.643</v>
+        <v>12744966.328</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>5965737.115</v>
+        <v>16070737.594</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1565,16 +1565,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>8885480.777000001</v>
+        <v>21278939.735</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>10923692.194</v>
+        <v>24473117.611</v>
       </c>
       <c r="Q9" t="n">
-        <v>11287538.739</v>
+        <v>25748136.107</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1687,13 +1687,13 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>5341911.006</v>
+        <v>15659104.044</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>19315754.459</v>
+        <v>44217984.188</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1708,10 +1708,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>11234613.437</v>
+        <v>28381164.148</v>
       </c>
       <c r="Q10" t="n">
-        <v>9284653.771</v>
+        <v>23988990.942</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1723,10 +1723,10 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>17246111.729</v>
+        <v>40501765.454</v>
       </c>
       <c r="V10" t="n">
-        <v>26220602.194</v>
+        <v>54958613.169</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -1827,7 +1827,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>11567162.042</v>
+        <v>26454038.715</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -1863,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>27046672.051</v>
+        <v>50722193.391</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>9775222.384</v>
+        <v>23470216.614</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -1988,10 +1988,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>10472449.158</v>
+        <v>23085448.641</v>
       </c>
       <c r="S12" t="n">
-        <v>13960677.761</v>
+        <v>27151291.106</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -2092,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>6534473.007</v>
+        <v>15784427.902</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -2116,7 +2116,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>6484911.455</v>
+        <v>17189734.179</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -2128,7 +2128,7 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>11090227.769</v>
+        <v>24960323.752</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5427848.161</v>
+        <v>16936531.862</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -2253,10 +2253,10 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>7790816.599</v>
+        <v>21627906.03</v>
       </c>
       <c r="P14" t="n">
-        <v>8975228.963</v>
+        <v>24384935.009</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -2387,13 +2387,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>3771438.312</v>
+        <v>10966608.059</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>8894438.436000001</v>
+        <v>21771987.533</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -2405,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>13124905.624</v>
+        <v>28443880.994</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>20982900.717</v>
+        <v>41801334.642</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -2533,7 +2533,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>6288574.633</v>
+        <v>16079398.035</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -2545,7 +2545,7 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>12344581.731</v>
+        <v>25297804.314</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
@@ -2554,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>18159647.818</v>
+        <v>36229621.513</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -2682,7 +2682,7 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>8495935.429</v>
+        <v>19227268.788</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -2813,7 +2813,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>8801282.557</v>
+        <v>21220721.149</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -2932,13 +2932,13 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>5227002.481</v>
+        <v>16651106.01</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>10913107.797</v>
+        <v>28243241.037</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -2953,7 +2953,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>6651378.626</v>
+        <v>18683751.916</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -3075,7 +3075,7 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>7070702.592</v>
+        <v>17713568.353</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -3087,22 +3087,22 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>3473528.167</v>
+        <v>10192077.756</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>15571488.382</v>
+        <v>33305146.67</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>15310138.6</v>
+        <v>30290841.445</v>
       </c>
       <c r="X20" t="n">
-        <v>14588274.417</v>
+        <v>30509737.959</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -3239,16 +3239,16 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>14951711.211</v>
+        <v>35425920.34</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>12777354.246</v>
+        <v>30579770.908</v>
       </c>
       <c r="AA21" t="n">
-        <v>25659160.493</v>
+        <v>57037024.255</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>
@@ -3302,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>16606349.112</v>
+        <v>38834598.098</v>
       </c>
     </row>
     <row r="22">
@@ -3367,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>7530702.863</v>
+        <v>21235278.127</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -3382,7 +3382,7 @@
         <v>0</v>
       </c>
       <c r="Z22" t="n">
-        <v>14500828.738</v>
+        <v>31187130.514</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
@@ -3501,10 +3501,10 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>7974339.159</v>
+        <v>18070278.903</v>
       </c>
       <c r="U23" t="n">
-        <v>19747328.541</v>
+        <v>39131526.526</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>10922632.506</v>
+        <v>22851984.854</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -3641,7 +3641,7 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>12541828.081</v>
+        <v>31457077.867</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -3653,7 +3653,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>5346379.34</v>
+        <v>16007361.023</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
@@ -3787,16 +3787,16 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>3019274.436</v>
+        <v>9963152.275</v>
       </c>
       <c r="Y25" t="n">
         <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>17371958.526</v>
+        <v>40442621.586</v>
       </c>
       <c r="AA25" t="n">
-        <v>16862932.58</v>
+        <v>37435978.757</v>
       </c>
       <c r="AB25" t="n">
         <v>0</v>
@@ -3850,7 +3850,7 @@
         <v>0</v>
       </c>
       <c r="AS25" t="n">
-        <v>17010654.819</v>
+        <v>38569332.94</v>
       </c>
     </row>
     <row r="26">
@@ -3927,7 +3927,7 @@
         <v>0</v>
       </c>
       <c r="Y26" t="n">
-        <v>14419978.42</v>
+        <v>31533840.327</v>
       </c>
       <c r="Z26" t="n">
         <v>0</v>
@@ -3936,13 +3936,13 @@
         <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>11887336.562</v>
+        <v>26394919.855</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>20135237.566</v>
+        <v>42314653.738</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -3987,7 +3987,7 @@
         <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>6286914.042</v>
+        <v>17341318.164</v>
       </c>
     </row>
     <row r="27">
@@ -4073,28 +4073,28 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>18226518.646</v>
+        <v>37853238.431</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>16195261.047</v>
+        <v>34407444.573</v>
       </c>
       <c r="AE27" t="n">
-        <v>23013899.923</v>
+        <v>47267818.899</v>
       </c>
       <c r="AF27" t="n">
-        <v>14736605.761</v>
+        <v>31211039.233</v>
       </c>
       <c r="AG27" t="n">
-        <v>14468978.655</v>
+        <v>31083590.453</v>
       </c>
       <c r="AH27" t="n">
         <v>0</v>
       </c>
       <c r="AI27" t="n">
-        <v>17571312.2</v>
+        <v>36152091.587</v>
       </c>
       <c r="AJ27" t="n">
         <v>0</v>
@@ -4124,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="AS27" t="n">
-        <v>13900223.769</v>
+        <v>30262259.733</v>
       </c>
     </row>
     <row r="28">
@@ -4207,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="AA28" t="n">
-        <v>15922645.239</v>
+        <v>33929742.998</v>
       </c>
       <c r="AB28" t="n">
         <v>0</v>
@@ -4216,10 +4216,10 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>11723950.81</v>
+        <v>26060428.985</v>
       </c>
       <c r="AE28" t="n">
-        <v>12095805.123</v>
+        <v>25462334.791</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
@@ -4344,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>42863877.014</v>
+        <v>74611728.858</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -4365,10 +4365,10 @@
         <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>30631832.97</v>
+        <v>53831949.516</v>
       </c>
       <c r="AI29" t="n">
-        <v>41321354.793</v>
+        <v>73148418.499</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -4493,13 +4493,13 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>9645032.526000001</v>
+        <v>21284412.087</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
       </c>
       <c r="AG30" t="n">
-        <v>5653504.381</v>
+        <v>15111026.766</v>
       </c>
       <c r="AH30" t="n">
         <v>0</v>
@@ -4508,13 +4508,13 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>17656215.019</v>
+        <v>37324103.938</v>
       </c>
       <c r="AK30" t="n">
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>15413974.664</v>
+        <v>33043120.993</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
@@ -4627,7 +4627,7 @@
         <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>8414252.550000001</v>
+        <v>19153696.525</v>
       </c>
       <c r="AE31" t="n">
         <v>0</v>
@@ -4645,13 +4645,13 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>15002116.384</v>
+        <v>31751557.854</v>
       </c>
       <c r="AK31" t="n">
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>13850255.241</v>
+        <v>30172036.445</v>
       </c>
       <c r="AM31" t="n">
         <v>0</v>
@@ -4773,13 +4773,13 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
-        <v>6035405.064</v>
+        <v>17059324.003</v>
       </c>
       <c r="AH32" t="n">
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>7815207.91</v>
+        <v>20057588.837</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -4788,7 +4788,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>21383688.006</v>
+        <v>48562664.182</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -4901,13 +4901,13 @@
         <v>0</v>
       </c>
       <c r="AD33" t="n">
-        <v>5218473.715</v>
+        <v>13940183.318</v>
       </c>
       <c r="AE33" t="n">
         <v>0</v>
       </c>
       <c r="AF33" t="n">
-        <v>5223805.445</v>
+        <v>13956063.272</v>
       </c>
       <c r="AG33" t="n">
         <v>0</v>
@@ -4925,7 +4925,7 @@
         <v>0</v>
       </c>
       <c r="AL33" t="n">
-        <v>17221705.652</v>
+        <v>35289386.884</v>
       </c>
       <c r="AM33" t="n">
         <v>0</v>
@@ -5053,19 +5053,19 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
-        <v>14840099.291</v>
+        <v>32745698.132</v>
       </c>
       <c r="AJ34" t="n">
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>9077992.708000001</v>
+        <v>20356184.891</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
       </c>
       <c r="AM34" t="n">
-        <v>16428666.588</v>
+        <v>35942124.532</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -5181,7 +5181,7 @@
         <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>5364717.35</v>
+        <v>14311405.679</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -5202,7 +5202,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="n">
-        <v>10265354.688</v>
+        <v>23220207.128</v>
       </c>
       <c r="AN35" t="n">
         <v>0</v>
@@ -5336,7 +5336,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>5628128.291</v>
+        <v>14910239.647</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -5345,7 +5345,7 @@
         <v>0</v>
       </c>
       <c r="AO36" t="n">
-        <v>16696109.511</v>
+        <v>0</v>
       </c>
       <c r="AP36" t="n">
         <v>0</v>
@@ -5461,10 +5461,10 @@
         <v>0</v>
       </c>
       <c r="AH37" t="n">
-        <v>6209624.441</v>
+        <v>14786172.722</v>
       </c>
       <c r="AI37" t="n">
-        <v>13689891.675</v>
+        <v>29048097.177</v>
       </c>
       <c r="AJ37" t="n">
         <v>0</v>
@@ -5476,7 +5476,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="n">
-        <v>12719385.223</v>
+        <v>26656339.891</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -5625,7 +5625,7 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
-        <v>5186532.415</v>
+        <v>15471903.293</v>
       </c>
       <c r="AR38" t="n">
         <v>0</v>
@@ -5738,7 +5738,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="n">
-        <v>6597327.838</v>
+        <v>16082792.229</v>
       </c>
       <c r="AJ39" t="n">
         <v>0</v>
@@ -5881,13 +5881,13 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
-        <v>17544317.781</v>
+        <v>38168577.422</v>
       </c>
       <c r="AL40" t="n">
         <v>0</v>
       </c>
       <c r="AM40" t="n">
-        <v>21273343.257</v>
+        <v>46330025.603</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -6021,7 +6021,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>15185780.988</v>
+        <v>31392054.327</v>
       </c>
       <c r="AM41" t="n">
         <v>0</v>
@@ -6155,13 +6155,13 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
-        <v>26070312.183</v>
+        <v>52667250.055</v>
       </c>
       <c r="AL42" t="n">
         <v>0</v>
       </c>
       <c r="AM42" t="n">
-        <v>23700399.371</v>
+        <v>48637206.882</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
@@ -6313,7 +6313,7 @@
         <v>0</v>
       </c>
       <c r="AR43" t="n">
-        <v>3042015.556</v>
+        <v>0</v>
       </c>
       <c r="AS43" t="n">
         <v>0</v>
@@ -6533,19 +6533,19 @@
         <v>0</v>
       </c>
       <c r="Z45" t="n">
-        <v>5441450.231</v>
+        <v>14462315.458</v>
       </c>
       <c r="AA45" t="n">
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>9687115.025</v>
+        <v>20905444.884</v>
       </c>
       <c r="AC45" t="n">
         <v>0</v>
       </c>
       <c r="AD45" t="n">
-        <v>15950315.116</v>
+        <v>33107662.378</v>
       </c>
       <c r="AE45" t="n">
         <v>0</v>
@@ -6752,7 +6752,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>396836.255</v>
+        <v>91758.05</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -6910,7 +6910,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>676760.808</v>
+        <v>128734.902</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -7038,13 +7038,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>223685.926</v>
+        <v>81427.056</v>
       </c>
       <c r="I4" t="n">
-        <v>200033.479</v>
+        <v>78626.535</v>
       </c>
       <c r="J4" t="n">
-        <v>242224.784</v>
+        <v>82199.867</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -7169,7 +7169,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>176842.288</v>
+        <v>60225.772</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -7187,10 +7187,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>304159.013</v>
+        <v>77162.056</v>
       </c>
       <c r="M5" t="n">
-        <v>341784.483</v>
+        <v>87139.57399999999</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -7309,7 +7309,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>215126.677</v>
+        <v>70674.158</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -7324,10 +7324,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>251775.852</v>
+        <v>70715.98</v>
       </c>
       <c r="M6" t="n">
-        <v>284064.136</v>
+        <v>79650.39</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -7449,7 +7449,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>170867.185</v>
+        <v>62966.587</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -7464,10 +7464,10 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>249986.237</v>
+        <v>73849.318</v>
       </c>
       <c r="N7" t="n">
-        <v>231461.651</v>
+        <v>67539.62</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -7583,13 +7583,13 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>139835.638</v>
+        <v>58254.037</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>174787.935</v>
+        <v>63505.834</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -7604,16 +7604,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>217472.309</v>
+        <v>67932.69</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>239420.551</v>
+        <v>78019.83900000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>256304.465</v>
+        <v>83916.85000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -7723,13 +7723,13 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>153257.355</v>
+        <v>58404.298</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>167892.99</v>
+        <v>64751.862</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -7741,16 +7741,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>205091.481</v>
+        <v>72716.429</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>227076.685</v>
+        <v>77442.891</v>
       </c>
       <c r="Q9" t="n">
-        <v>232682.486</v>
+        <v>79688.268</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -7863,13 +7863,13 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>151975.818</v>
+        <v>60813.532</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>379760.435</v>
+        <v>86719.368</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -7884,10 +7884,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>233404.831</v>
+        <v>78253.76300000001</v>
       </c>
       <c r="Q10" t="n">
-        <v>212235.556</v>
+        <v>74606.541</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -7899,10 +7899,10 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>319952.724</v>
+        <v>92061.249</v>
       </c>
       <c r="V10" t="n">
-        <v>444151.591</v>
+        <v>102136.535</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -8003,7 +8003,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>242960.938</v>
+        <v>83922.226</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -8039,7 +8039,7 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>497371.661</v>
+        <v>102882.883</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -8149,7 +8149,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>332512.107</v>
+        <v>72593.427</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -8164,10 +8164,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>288184.843</v>
+        <v>71743.459</v>
       </c>
       <c r="S12" t="n">
-        <v>305926.415</v>
+        <v>79166.639</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -8268,7 +8268,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>154168.234</v>
+        <v>64268.775</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -8292,7 +8292,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>266135.957</v>
+        <v>68595.49800000001</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -8304,7 +8304,7 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>319638.71</v>
+        <v>74325.145</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -8408,7 +8408,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>161661.065</v>
+        <v>60064.483</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -8429,10 +8429,10 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>270786.575</v>
+        <v>67483.019</v>
       </c>
       <c r="P14" t="n">
-        <v>254905.38</v>
+        <v>67419.90700000001</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -8563,13 +8563,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>141530.392</v>
+        <v>57492.597</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>278679.533</v>
+        <v>70370.77499999999</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -8581,7 +8581,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>275039.345</v>
+        <v>75257.49000000001</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -8593,7 +8593,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>381365.795</v>
+        <v>102488.15</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -8709,7 +8709,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>186910.71</v>
+        <v>67194.817</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -8721,7 +8721,7 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>251513.631</v>
+        <v>86278.55100000001</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
@@ -8730,7 +8730,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>351062.91</v>
+        <v>101548.105</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -8858,7 +8858,7 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>181067.282</v>
+        <v>70713.618</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -8989,7 +8989,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>286108.794</v>
+        <v>69998.38400000001</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -9108,13 +9108,13 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>163654.392</v>
+        <v>59753.364</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>294160.571</v>
+        <v>70365.421</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -9129,7 +9129,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>236369.709</v>
+        <v>64001.165</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -9251,7 +9251,7 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>159526.24</v>
+        <v>65328.729</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -9263,22 +9263,22 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>132736.25</v>
+        <v>56219.297</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>323337.953</v>
+        <v>94690.977</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>299034.074</v>
+        <v>80204.81299999999</v>
       </c>
       <c r="X20" t="n">
-        <v>302925.872</v>
+        <v>84462.874</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -9415,16 +9415,16 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>300346.43</v>
+        <v>90748.696</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>275595.844</v>
+        <v>85897.75999999999</v>
       </c>
       <c r="AA21" t="n">
-        <v>435008.9</v>
+        <v>119879.681</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>
@@ -9478,7 +9478,7 @@
         <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>310322.394</v>
+        <v>96412.89599999999</v>
       </c>
     </row>
     <row r="22">
@@ -9543,7 +9543,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>248070.676</v>
+        <v>66242.489</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -9558,7 +9558,7 @@
         <v>0</v>
       </c>
       <c r="Z22" t="n">
-        <v>273099.537</v>
+        <v>78767.959</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
@@ -9677,10 +9677,10 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>168587.082</v>
+        <v>70106.698</v>
       </c>
       <c r="U23" t="n">
-        <v>347201.175</v>
+        <v>104167.179</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -9689,7 +9689,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>266646.859</v>
+        <v>74065.05899999999</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -9817,7 +9817,7 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>256733.485</v>
+        <v>85560.58</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -9829,7 +9829,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>225775.014</v>
+        <v>64494.82</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
@@ -9963,16 +9963,16 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>135586.899</v>
+        <v>55912.657</v>
       </c>
       <c r="Y25" t="n">
         <v>0</v>
       </c>
       <c r="Z25" t="n">
-        <v>324566.089</v>
+        <v>97120.34600000001</v>
       </c>
       <c r="AA25" t="n">
-        <v>342708.225</v>
+        <v>88347.264</v>
       </c>
       <c r="AB25" t="n">
         <v>0</v>
@@ -10026,7 +10026,7 @@
         <v>0</v>
       </c>
       <c r="AS25" t="n">
-        <v>315423.399</v>
+        <v>93688.014</v>
       </c>
     </row>
     <row r="26">
@@ -10103,7 +10103,7 @@
         <v>0</v>
       </c>
       <c r="Y26" t="n">
-        <v>275936.202</v>
+        <v>93401.05</v>
       </c>
       <c r="Z26" t="n">
         <v>0</v>
@@ -10112,13 +10112,13 @@
         <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>248859.702</v>
+        <v>82533.75</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>364919.482</v>
+        <v>112553.684</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -10163,7 +10163,7 @@
         <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>193229.253</v>
+        <v>66333.999</v>
       </c>
     </row>
     <row r="27">
@@ -10249,28 +10249,28 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>325434.931</v>
+        <v>104050.32</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>318693.35</v>
+        <v>98346.515</v>
       </c>
       <c r="AE27" t="n">
-        <v>411300.821</v>
+        <v>118451.711</v>
       </c>
       <c r="AF27" t="n">
-        <v>300326.36</v>
+        <v>90541.42999999999</v>
       </c>
       <c r="AG27" t="n">
-        <v>284856.764</v>
+        <v>93163.788</v>
       </c>
       <c r="AH27" t="n">
         <v>0</v>
       </c>
       <c r="AI27" t="n">
-        <v>342066.528</v>
+        <v>97535.11</v>
       </c>
       <c r="AJ27" t="n">
         <v>0</v>
@@ -10300,7 +10300,7 @@
         <v>0</v>
       </c>
       <c r="AS27" t="n">
-        <v>291864.947</v>
+        <v>90522.912</v>
       </c>
     </row>
     <row r="28">
@@ -10383,7 +10383,7 @@
         <v>0</v>
       </c>
       <c r="AA28" t="n">
-        <v>288320.936</v>
+        <v>97998.43799999999</v>
       </c>
       <c r="AB28" t="n">
         <v>0</v>
@@ -10392,10 +10392,10 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>246328.323</v>
+        <v>86138.408</v>
       </c>
       <c r="AE28" t="n">
-        <v>234014.031</v>
+        <v>79810.41899999999</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
@@ -10520,7 +10520,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>691020.8100000001</v>
+        <v>135112.988</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -10541,10 +10541,10 @@
         <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>494395.23</v>
+        <v>110023.916</v>
       </c>
       <c r="AI29" t="n">
-        <v>664412.25</v>
+        <v>138130.54</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -10669,13 +10669,13 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>211175.566</v>
+        <v>78469.757</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
       </c>
       <c r="AG30" t="n">
-        <v>174063.459</v>
+        <v>65433.618</v>
       </c>
       <c r="AH30" t="n">
         <v>0</v>
@@ -10684,13 +10684,13 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>330174.219</v>
+        <v>105542.607</v>
       </c>
       <c r="AK30" t="n">
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>305286.359</v>
+        <v>98410.531</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
@@ -10803,7 +10803,7 @@
         <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>186278.964</v>
+        <v>73503.757</v>
       </c>
       <c r="AE31" t="n">
         <v>0</v>
@@ -10821,13 +10821,13 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>293208.677</v>
+        <v>92801.117</v>
       </c>
       <c r="AK31" t="n">
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>280969.489</v>
+        <v>91546.08199999999</v>
       </c>
       <c r="AM31" t="n">
         <v>0</v>
@@ -10949,13 +10949,13 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
-        <v>186156.717</v>
+        <v>64671.107</v>
       </c>
       <c r="AH32" t="n">
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>212238.573</v>
+        <v>67006.74800000001</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -10964,7 +10964,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>386527.229</v>
+        <v>113609.848</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -11077,13 +11077,13 @@
         <v>0</v>
       </c>
       <c r="AD33" t="n">
-        <v>161153.811</v>
+        <v>62126.383</v>
       </c>
       <c r="AE33" t="n">
         <v>0</v>
       </c>
       <c r="AF33" t="n">
-        <v>163611.695</v>
+        <v>62200.099</v>
       </c>
       <c r="AG33" t="n">
         <v>0</v>
@@ -11101,7 +11101,7 @@
         <v>0</v>
       </c>
       <c r="AL33" t="n">
-        <v>309869.527</v>
+        <v>104407.672</v>
       </c>
       <c r="AM33" t="n">
         <v>0</v>
@@ -11229,19 +11229,19 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
-        <v>299817.779</v>
+        <v>86679.27899999999</v>
       </c>
       <c r="AJ34" t="n">
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>205147.596</v>
+        <v>69937.83900000001</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
       </c>
       <c r="AM34" t="n">
-        <v>332903.751</v>
+        <v>89524.818</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -11357,7 +11357,7 @@
         <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>152231.264</v>
+        <v>61563.036</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -11378,7 +11378,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="n">
-        <v>240014.866</v>
+        <v>72409.234</v>
       </c>
       <c r="AN35" t="n">
         <v>0</v>
@@ -11512,7 +11512,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>168505.557</v>
+        <v>64864.063</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -11521,7 +11521,7 @@
         <v>0</v>
       </c>
       <c r="AO36" t="n">
-        <v>343878.465</v>
+        <v>0</v>
       </c>
       <c r="AP36" t="n">
         <v>0</v>
@@ -11637,10 +11637,10 @@
         <v>0</v>
       </c>
       <c r="AH37" t="n">
-        <v>147428.998</v>
+        <v>64346.834</v>
       </c>
       <c r="AI37" t="n">
-        <v>279344.437</v>
+        <v>87847.246</v>
       </c>
       <c r="AJ37" t="n">
         <v>0</v>
@@ -11652,7 +11652,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="n">
-        <v>259417.902</v>
+        <v>80013.78200000001</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -11801,7 +11801,7 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
-        <v>170390.846</v>
+        <v>62376.046</v>
       </c>
       <c r="AR38" t="n">
         <v>0</v>
@@ -11914,7 +11914,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="n">
-        <v>162309.229</v>
+        <v>65037.762</v>
       </c>
       <c r="AJ39" t="n">
         <v>0</v>
@@ -12057,13 +12057,13 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
-        <v>359509.47</v>
+        <v>87811.016</v>
       </c>
       <c r="AL40" t="n">
         <v>0</v>
       </c>
       <c r="AM40" t="n">
-        <v>370480.205</v>
+        <v>106670.465</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -12197,7 +12197,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>308187.102</v>
+        <v>91293.594</v>
       </c>
       <c r="AM41" t="n">
         <v>0</v>
@@ -12331,13 +12331,13 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
-        <v>438126.995</v>
+        <v>127081.526</v>
       </c>
       <c r="AL42" t="n">
         <v>0</v>
       </c>
       <c r="AM42" t="n">
-        <v>402027.944</v>
+        <v>121735.992</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
       <c r="AR43" t="n">
-        <v>213074.604</v>
+        <v>13273.625</v>
       </c>
       <c r="AS43" t="n">
         <v>0</v>
@@ -12709,19 +12709,19 @@
         <v>0</v>
       </c>
       <c r="Z45" t="n">
-        <v>169474.854</v>
+        <v>63025.866</v>
       </c>
       <c r="AA45" t="n">
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>211820.732</v>
+        <v>78983.13099999999</v>
       </c>
       <c r="AC45" t="n">
         <v>0</v>
       </c>
       <c r="AD45" t="n">
-        <v>300453.543</v>
+        <v>100160.418</v>
       </c>
       <c r="AE45" t="n">
         <v>0</v>

</xml_diff>